<commit_message>
wirelist xlsx: wrap long columns, frozen bold 12pt header with dark underline, FROM blue / TO green group tints, 80% zoom, filters, landscape (Dan 2026-10-19)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/A-cabin-pinouts.xlsx
+++ b/docs/harness/wirelist/A-cabin-pinouts.xlsx
@@ -14,7 +14,20 @@
     <sheet name="+5V BUS bus_5v_bha_p" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="SENSOR GND BUS bus_gnd_bha_p" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ECU-A ecu_a'!$A$2:$D$36</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'ECU-A ecu_a'!$2:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BULKHEAD bh_a_fw'!$A$2:$D$51</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'BULKHEAD bh_a_fw'!$2:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'FRONT WS INLINE ix_ws_front_p'!$A$2:$D$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'FRONT WS INLINE ix_ws_front_p'!$2:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PEDAL aps'!$A$2:$D$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'PEDAL aps'!$2:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'+5V BUS bus_5v_bha_p'!$A$2:$D$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'+5V BUS bus_5v_bha_p'!$2:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'SENSOR GND BUS bus_gnd_bha_p'!$A$2:$D$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'SENSOR GND BUS bus_gnd_bha_p'!$2:$2</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -22,7 +35,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,7 +45,15 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F1F1F"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="11">
@@ -44,22 +65,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0044546A"/>
+        <fgColor rgb="00BFBFBF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E0E0E0"/>
+        <fgColor rgb="00F8F8F8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="009DC3E6"/>
       </patternFill>
     </fill>
     <fill>
@@ -69,26 +90,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
+        <fgColor rgb="00EEF5FB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C55A11"/>
+        <fgColor rgb="00A9D18E"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00E2F0D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8CBAD"/>
+        <fgColor rgb="00F1F8EC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -97,44 +118,63 @@
       <diagonal/>
     </border>
     <border>
+      <bottom style="thick">
+        <color rgb="001F1F1F"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="hair">
+        <color rgb="00A6A6A6"/>
+      </bottom>
+    </border>
+    <border>
       <left style="thin">
-        <color rgb="00FFFFFF"/>
+        <color rgb="00404040"/>
       </left>
-      <right style="thin">
-        <color rgb="00FFFFFF"/>
-      </right>
+      <bottom style="thick">
+        <color rgb="001F1F1F"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00404040"/>
+      </left>
+      <bottom style="hair">
+        <color rgb="00A6A6A6"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -211,84 +251,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Pinout1" displayName="Pinout1" ref="A1:D35" headerRowCount="1">
-  <autoFilter ref="A1:D35"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Pin"/>
-    <tableColumn id="2" name="Wire"/>
-    <tableColumn id="3" name="Description"/>
-    <tableColumn id="4" name="Other end"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Pinout2" displayName="Pinout2" ref="A1:D50" headerRowCount="1">
-  <autoFilter ref="A1:D50"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Pin"/>
-    <tableColumn id="2" name="Wire"/>
-    <tableColumn id="3" name="Description"/>
-    <tableColumn id="4" name="Other end"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Pinout3" displayName="Pinout3" ref="A1:D7" headerRowCount="1">
-  <autoFilter ref="A1:D7"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Pin"/>
-    <tableColumn id="2" name="Wire"/>
-    <tableColumn id="3" name="Description"/>
-    <tableColumn id="4" name="Other end"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Pinout4" displayName="Pinout4" ref="A1:D7" headerRowCount="1">
-  <autoFilter ref="A1:D7"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Pin"/>
-    <tableColumn id="2" name="Wire"/>
-    <tableColumn id="3" name="Description"/>
-    <tableColumn id="4" name="Other end"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Pinout5" displayName="Pinout5" ref="A1:D9" headerRowCount="1">
-  <autoFilter ref="A1:D9"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Pin"/>
-    <tableColumn id="2" name="Wire"/>
-    <tableColumn id="3" name="Description"/>
-    <tableColumn id="4" name="Other end"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Pinout6" displayName="Pinout6" ref="A1:D9" headerRowCount="1">
-  <autoFilter ref="A1:D9"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Pin"/>
-    <tableColumn id="2" name="Wire"/>
-    <tableColumn id="3" name="Description"/>
-    <tableColumn id="4" name="Other end"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -578,792 +540,798 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>ECU-A ecu_a</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>Pin</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Wire</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Other end</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>w111_c</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Injector 4 drive (-)</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 34</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>w110_c</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Injector 3 drive (-)</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 33</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>w109_c</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Injector 2 drive (-)</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 32</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>A4</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>w108_c</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Injector 1 drive (-)</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 31</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>A5</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>w78</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>ECU main +12 V</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>splice sp_sw12 (SP-SW12: switched +12 V)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>A6</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>w19</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>+8 V sensor supply</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>splice sp_8v (SP-8V: +8 V cam sensor supply)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>A7</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>w_drain_ecu_a</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Shield drain</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>A8</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>w200_c</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Crank sensor signal</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 9</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>A9</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>w_trig2_pin</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Cam sensor signal</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>splice sp_trig2 (SP-CAM: cam signal + 1.8k pull-up to +8V)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>A10</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>w123_c</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>Coil 4 trigger (IGT)</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 38</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>A11</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>w122_c</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Coil 3 trigger (IGT)</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 37</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>A12</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>w121_c</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>Coil 2 trigger (IGT)</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 36</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>A13</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>w120_c</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Coil 1 trigger (IGT)</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 35</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>A14</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>w38</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>Pedal 1 signal main</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>PEDAL pin 6</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>A15</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>w201_c</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Coolant temp signal</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 40</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>A16</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>w202_c</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>Intake temp signal</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 41</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>A17</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>w26_c</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>MAP sensor signal</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 30</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>A18</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>w_ac_kill</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>A/C cancel (ACT)</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>OEM A/C amplifier pin 11</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>A19</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>w_fp85</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Fuel pump relay (-)</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>FP RELAY K1 pin 85</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>A20</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>w81</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>ETB relay coil (-)</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D22" s="10" t="inlineStr">
         <is>
           <t>LOGIC M4 pin 85</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>A21</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>w103_c</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Boost solenoid (-)</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 39</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>A22</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>w128_c</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>Throttle pos 1 main</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 24</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>A23</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>cab_fspur_l</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>FL conditioned out</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>FRONT WS INLINE pin 3</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>A24</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>w68</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>Sensor ground</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D26" s="10" t="inlineStr">
         <is>
           <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>A25</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>w70</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>ECU power ground</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>splice sp_chassis (SP-GND-CHASSIS: ECU power ground)</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>A26</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>w_str85</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>Start relay coil (-)</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D28" s="10" t="inlineStr">
         <is>
           <t>POWER R3 pin 85</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>A27</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>w_mrs_c</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>EHPS pump speed</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 44</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>A28</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>w76</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>EFI relay coil (-)</t>
         </is>
       </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="D30" s="10" t="inlineStr">
         <is>
           <t>POWER R2 pin 85</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>A29</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>w_fan85</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>Rad fan relay (-)</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>POWER R4 pin 85</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="7" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>A30</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>w16_c</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>Turbo speed signal</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D32" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 17</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>A31</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>w48_c</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>Flex fuel signal</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 21</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="7" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>A32</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>w67</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>+5 V sensor supply</t>
         </is>
       </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="D34" s="10" t="inlineStr">
         <is>
           <t>splice sp_5v (SP-5V-A: +5 V sensor supply)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>A33</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>w129_c</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>Throttle pos 2 sub</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 25</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="7" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>A34</t>
         </is>
       </c>
-      <c r="B35" s="7" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>w_a34</t>
         </is>
       </c>
-      <c r="C35" s="8" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>ECU power ground</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D36" s="10" t="inlineStr">
         <is>
           <t>splice sp_chassis (SP-GND-CHASSIS: ECU power ground)</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A2:D36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1371,960 +1339,966 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>BULKHEAD bh_a_fw</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>Pin</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Wire</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Other end</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="n">
+    <row r="3">
+      <c r="A3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>w_inj_pwr_ac</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Injector +12 V feed</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>FB-LOGIC pin BUS2-4</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="7" t="n">
+    <row r="4">
+      <c r="A4" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>w_cop_pwr_ac</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Coil +12 V feed</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>FB-LOGIC pin BUS2-3</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
+    <row r="5">
+      <c r="A5" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>w200_c</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Crank sensor signal</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A8</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+    <row r="6">
+      <c r="A6" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>w_gnd_a_c41</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Gnd crank sensor</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>SENSOR GND BUS pin 3</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>w_shc_crank</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Crank sensor shield</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+    <row r="8">
+      <c r="A8" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>w_rail_sp_8v_c</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>+8 V to cam sensor</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>splice sp_8v (SP-8V: +8 V cam sensor supply)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
+    <row r="9">
+      <c r="A9" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>w_cam_sig_c</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Cam sensor signal</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>splice sp_trig2 (SP-CAM: cam signal + 1.8k pull-up to +8V)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="n">
+    <row r="10">
+      <c r="A10" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>w_gnd_a_c42</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Gnd cam sensor</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>SENSOR GND BUS pin 4</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
+    <row r="11">
+      <c r="A11" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>w_shc_cam</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Cam sensor shield</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="n">
+    <row r="12">
+      <c r="A12" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>w_5v_a_c40</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>+5 V turbo speed</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>+5V BUS pin 4</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
+    <row r="13">
+      <c r="A13" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>w16_c</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Turbo speed signal</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A30</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="7" t="n">
+    <row r="14">
+      <c r="A14" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>w_gnd_a_c43</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>Gnd turbo speed</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>SENSOR GND BUS pin 5</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="n">
+    <row r="15">
+      <c r="A15" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>w_shc_turbo</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Turbo speed shield</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="n">
+    <row r="16">
+      <c r="A16" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>w_rail_sp_sw12_c</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>+12 V boost + flex</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>splice sp_sw12 (SP-SW12: switched +12 V)</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
+    <row r="17">
+      <c r="A17" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>w48_c</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Flex fuel signal</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A31</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="7" t="n">
+    <row r="18">
+      <c r="A18" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>w_shc_flex</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>Flex fuel shield</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
+    <row r="19">
+      <c r="A19" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>w_rail_sp_5v_c</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>+5 V throttle sensor</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>+5V BUS pin 2</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="7" t="n">
+    <row r="20">
+      <c r="A20" s="8" t="n">
         <v>24</v>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>w128_c</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>Throttle pos 1 main</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>ECU-A pin A22</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
+    <row r="21">
+      <c r="A21" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>w129_c</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Throttle pos 2 sub</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A33</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="7" t="n">
+    <row r="22">
+      <c r="A22" s="8" t="n">
         <v>26</v>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>w_rail_sp_gndout_c</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>Gnd IAT/TPS/coolant</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D22" s="10" t="inlineStr">
         <is>
           <t>SENSOR GND BUS pin 2</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="n">
+    <row r="23">
+      <c r="A23" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>w_shc_etbs</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Throttle shield</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="7" t="n">
+    <row r="24">
+      <c r="A24" s="8" t="n">
         <v>28</v>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>w_5v_a_c39</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>+5 V MAP sensor</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>+5V BUS pin 3</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="n">
+    <row r="25">
+      <c r="A25" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>w_gnd_a_c44</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>Gnd flex + MAP</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>SENSOR GND BUS pin 6</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="7" t="n">
+    <row r="26">
+      <c r="A26" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>w26_c</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>MAP sensor signal</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D26" s="10" t="inlineStr">
         <is>
           <t>ECU-A pin A17</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="n">
+    <row r="27">
+      <c r="A27" s="5" t="n">
         <v>31</v>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>w108_c</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>Injector 1 drive (-)</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A4</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="7" t="n">
+    <row r="28">
+      <c r="A28" s="8" t="n">
         <v>32</v>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>w109_c</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>Injector 2 drive (-)</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D28" s="10" t="inlineStr">
         <is>
           <t>ECU-A pin A3</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="n">
+    <row r="29">
+      <c r="A29" s="5" t="n">
         <v>33</v>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>w110_c</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>Injector 3 drive (-)</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A2</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="7" t="n">
+    <row r="30">
+      <c r="A30" s="8" t="n">
         <v>34</v>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>w111_c</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>Injector 4 drive (-)</t>
         </is>
       </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="D30" s="10" t="inlineStr">
         <is>
           <t>ECU-A pin A1</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="n">
+    <row r="31">
+      <c r="A31" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>w120_c</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>Coil 1 trigger (IGT)</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A13</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="7" t="n">
+    <row r="32">
+      <c r="A32" s="8" t="n">
         <v>36</v>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>w121_c</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>Coil 2 trigger (IGT)</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D32" s="10" t="inlineStr">
         <is>
           <t>ECU-A pin A12</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="n">
+    <row r="33">
+      <c r="A33" s="5" t="n">
         <v>37</v>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>w122_c</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>Coil 3 trigger (IGT)</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A11</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="7" t="n">
+    <row r="34">
+      <c r="A34" s="8" t="n">
         <v>38</v>
       </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>w123_c</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>Coil 4 trigger (IGT)</t>
         </is>
       </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="D34" s="10" t="inlineStr">
         <is>
           <t>ECU-A pin A10</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="n">
+    <row r="35">
+      <c r="A35" s="5" t="n">
         <v>39</v>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>w103_c</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>Boost solenoid (-)</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A21</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="7" t="n">
+    <row r="36">
+      <c r="A36" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="B35" s="7" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>w201_c</t>
         </is>
       </c>
-      <c r="C35" s="8" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>Coolant temp signal</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D36" s="10" t="inlineStr">
         <is>
           <t>ECU-A pin A15</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="n">
+    <row r="37">
+      <c r="A37" s="5" t="n">
         <v>41</v>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>w202_c</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>Intake temp signal</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A16</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="7" t="n">
+    <row r="38">
+      <c r="A38" s="8" t="n">
         <v>42</v>
       </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t>w_fb_mrs_en</t>
         </is>
       </c>
-      <c r="C37" s="8" t="inlineStr">
+      <c r="C38" s="9" t="inlineStr">
         <is>
           <t>EHPS enable +12 V</t>
         </is>
       </c>
-      <c r="D37" s="9" t="inlineStr">
+      <c r="D38" s="10" t="inlineStr">
         <is>
           <t>FB-LOGIC pin BUS2-12</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="n">
+    <row r="39">
+      <c r="A39" s="5" t="n">
         <v>44</v>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>w_mrs_c</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>EHPS pump speed</t>
         </is>
       </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="D39" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A27</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="7" t="n">
+    <row r="40">
+      <c r="A40" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="B39" s="7" t="inlineStr"/>
-      <c r="C39" s="8" t="inlineStr">
+      <c r="B40" s="8" t="inlineStr"/>
+      <c r="C40" s="9" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D39" s="9" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="n">
+      <c r="D40" s="10" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="B40" s="4" t="inlineStr"/>
-      <c r="C40" s="5" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr"/>
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="7" t="n">
+      <c r="D41" s="7" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n">
         <v>47</v>
       </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="B42" s="8" t="inlineStr">
         <is>
           <t>w_5v_brail_c45</t>
         </is>
       </c>
-      <c r="C41" s="8" t="inlineStr">
+      <c r="C42" s="9" t="inlineStr">
         <is>
           <t>+5 V oil pressure</t>
         </is>
       </c>
-      <c r="D41" s="9" t="inlineStr">
+      <c r="D42" s="10" t="inlineStr">
         <is>
           <t>+5V BUS pin 5</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="4" t="n">
+    <row r="43">
+      <c r="A43" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="B42" s="4" t="inlineStr">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>w_5v_brail_c46</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>+5 V fuel pressure</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="D43" s="7" t="inlineStr">
         <is>
           <t>+5V BUS pin 6</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="7" t="n">
+    <row r="44">
+      <c r="A44" s="8" t="n">
         <v>51</v>
       </c>
-      <c r="B43" s="7" t="inlineStr">
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>w_5v_brail_c47</t>
         </is>
       </c>
-      <c r="C43" s="8" t="inlineStr">
+      <c r="C44" s="9" t="inlineStr">
         <is>
           <t>+5 V coolant press</t>
         </is>
       </c>
-      <c r="D43" s="9" t="inlineStr">
+      <c r="D44" s="10" t="inlineStr">
         <is>
           <t>+5V BUS pin 7</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="n">
+    <row r="45">
+      <c r="A45" s="5" t="n">
         <v>52</v>
       </c>
-      <c r="B44" s="4" t="inlineStr"/>
-      <c r="C44" s="5" t="inlineStr">
+      <c r="B45" s="5" t="inlineStr"/>
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D44" s="6" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="7" t="n">
+      <c r="D45" s="7" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="n">
         <v>53</v>
       </c>
-      <c r="B45" s="7" t="inlineStr"/>
-      <c r="C45" s="8" t="inlineStr">
+      <c r="B46" s="8" t="inlineStr"/>
+      <c r="C46" s="9" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D45" s="9" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="n">
+      <c r="D46" s="10" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="n">
         <v>56</v>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>w_eps_rly</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>EHPS relay coil (-)</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr">
+      <c r="D47" s="7" t="inlineStr">
         <is>
           <t>EHPS RELAY pin 85</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="7" t="n">
+    <row r="48">
+      <c r="A48" s="8" t="n">
         <v>57</v>
       </c>
-      <c r="B47" s="7" t="inlineStr"/>
-      <c r="C47" s="8" t="inlineStr">
+      <c r="B48" s="8" t="inlineStr"/>
+      <c r="C48" s="9" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D47" s="9" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="n">
+      <c r="D48" s="10" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="n">
         <v>58</v>
       </c>
-      <c r="B48" s="4" t="inlineStr"/>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr"/>
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D48" s="6" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="7" t="n">
+      <c r="D49" s="7" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="n">
         <v>59</v>
       </c>
-      <c r="B49" s="7" t="inlineStr"/>
-      <c r="C49" s="8" t="inlineStr">
+      <c r="B50" s="8" t="inlineStr"/>
+      <c r="C50" s="9" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D49" s="9" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="n">
+      <c r="D50" s="10" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="n">
         <v>61</v>
       </c>
-      <c r="B50" s="4" t="inlineStr"/>
-      <c r="C50" s="5" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr"/>
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D50" s="6" t="inlineStr"/>
+      <c r="D51" s="7" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A2:D51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2332,156 +2306,162 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>FRONT WS INLINE ix_ws_front_p</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>Pin</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Wire</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Other end</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="n">
+    <row r="3">
+      <c r="A3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>cab_fspur_5v</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>VRC-F +5V</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>splice sp_5v (SP-5V-A: +5 V sensor supply)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="7" t="n">
+    <row r="4">
+      <c r="A4" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>cab_fspur_gnd</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>VRC-F GND</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
+    <row r="5">
+      <c r="A5" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>cab_fspur_l</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>FL conditioned out</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A23</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+    <row r="6">
+      <c r="A6" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>cab_fspur_r_ac</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>FR conditioned out</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>ECU-B (Link G4X plug B, centre dash) pin B21</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>cab_fspur_sh</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>WS-F screen drain</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+    <row r="8">
+      <c r="A8" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr"/>
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr"/>
+      <c r="D8" s="10" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A2:D8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2489,164 +2469,170 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>PEDAL aps</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>Pin</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Wire</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Other end</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="n">
+    <row r="3">
+      <c r="A3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>w210</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>+5 V pedal sensor 2</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>splice sp_5v_2 (SP-5V-PEDAL: +5 V to pedal + cruise)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="7" t="n">
+    <row r="4">
+      <c r="A4" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>w_aps_gnd2</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Pedal 2 ground</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
+    <row r="5">
+      <c r="A5" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>w_aps_vpa2</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Pedal 2 signal sub</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>ECU-B (Link G4X plug B, centre dash) pin B33</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+    <row r="6">
+      <c r="A6" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>w_aps_vc1</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>+5 V pedal sensor 1</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>splice sp_5v_2 (SP-5V-PEDAL: +5 V to pedal + cruise)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>w40</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Pedal 1 ground</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+    <row r="8">
+      <c r="A8" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>w38</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Pedal 1 signal main</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>ECU-A pin A14</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A2:D8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2654,196 +2640,202 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>+5V BUS bus_5v_bha_p</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>Pin</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Wire</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Other end</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="n">
+    <row r="3">
+      <c r="A3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>w_5v_bha_trunk</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>+5 V sensor supply</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>splice sp_5v (SP-5V-A: +5 V sensor supply)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="7" t="n">
+    <row r="4">
+      <c r="A4" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>w_rail_sp_5v_c</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>+5 V throttle sensor</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 23</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
+    <row r="5">
+      <c r="A5" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>w_5v_a_c39</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>+5 V MAP sensor</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 28</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+    <row r="6">
+      <c r="A6" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>w_5v_a_c40</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>+5 V turbo speed</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 16</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>w_5v_brail_c45</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>+5 V oil pressure</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 47</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+    <row r="8">
+      <c r="A8" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>w_5v_brail_c46</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>+5 V fuel pressure</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 50</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
+    <row r="9">
+      <c r="A9" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>w_5v_brail_c47</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>+5 V coolant press</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 51</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="n">
+    <row r="10">
+      <c r="A10" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="inlineStr"/>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr"/>
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr"/>
+      <c r="D10" s="10" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A2:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2851,187 +2843,193 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>SENSOR GND BUS bus_gnd_bha_p</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>Pin</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Wire</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Other end</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="n">
+    <row r="3">
+      <c r="A3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>w_gnd_bha_trunk</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Sensor ground</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="7" t="n">
+    <row r="4">
+      <c r="A4" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>w_rail_sp_gndout_c</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Gnd IAT/TPS/coolant</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 26</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
+    <row r="5">
+      <c r="A5" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>w_gnd_a_c41</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Gnd crank sensor</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 10</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+    <row r="6">
+      <c r="A6" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>w_gnd_a_c42</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Gnd cam sensor</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 14</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>w_gnd_a_c43</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Gnd turbo speed</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 18</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+    <row r="8">
+      <c r="A8" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>w_gnd_a_c44</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Gnd flex + MAP</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 29</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
+    <row r="9">
+      <c r="A9" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="inlineStr"/>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr"/>
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="n">
+      <c r="D9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="inlineStr"/>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr"/>
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr"/>
+      <c r="D10" s="10" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A2:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
wirelist xlsx: wrap long columns, frozen bold 12pt header with dark underline, FROM blue / TO green group tints, 80% zoom, filters, landscape (Dan 2026-10-19) (#337)
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/A-cabin-pinouts.xlsx
+++ b/docs/harness/wirelist/A-cabin-pinouts.xlsx
@@ -14,7 +14,20 @@
     <sheet name="+5V BUS bus_5v_bha_p" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="SENSOR GND BUS bus_gnd_bha_p" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ECU-A ecu_a'!$A$2:$D$36</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'ECU-A ecu_a'!$2:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BULKHEAD bh_a_fw'!$A$2:$D$51</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'BULKHEAD bh_a_fw'!$2:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'FRONT WS INLINE ix_ws_front_p'!$A$2:$D$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'FRONT WS INLINE ix_ws_front_p'!$2:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PEDAL aps'!$A$2:$D$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'PEDAL aps'!$2:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'+5V BUS bus_5v_bha_p'!$A$2:$D$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'+5V BUS bus_5v_bha_p'!$2:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'SENSOR GND BUS bus_gnd_bha_p'!$A$2:$D$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'SENSOR GND BUS bus_gnd_bha_p'!$2:$2</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -22,7 +35,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,7 +45,15 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F1F1F"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="11">
@@ -44,22 +65,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0044546A"/>
+        <fgColor rgb="00BFBFBF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E0E0E0"/>
+        <fgColor rgb="00F8F8F8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="009DC3E6"/>
       </patternFill>
     </fill>
     <fill>
@@ -69,26 +90,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
+        <fgColor rgb="00EEF5FB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C55A11"/>
+        <fgColor rgb="00A9D18E"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00E2F0D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8CBAD"/>
+        <fgColor rgb="00F1F8EC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -97,44 +118,63 @@
       <diagonal/>
     </border>
     <border>
+      <bottom style="thick">
+        <color rgb="001F1F1F"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="hair">
+        <color rgb="00A6A6A6"/>
+      </bottom>
+    </border>
+    <border>
       <left style="thin">
-        <color rgb="00FFFFFF"/>
+        <color rgb="00404040"/>
       </left>
-      <right style="thin">
-        <color rgb="00FFFFFF"/>
-      </right>
+      <bottom style="thick">
+        <color rgb="001F1F1F"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00404040"/>
+      </left>
+      <bottom style="hair">
+        <color rgb="00A6A6A6"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -211,84 +251,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Pinout1" displayName="Pinout1" ref="A1:D35" headerRowCount="1">
-  <autoFilter ref="A1:D35"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Pin"/>
-    <tableColumn id="2" name="Wire"/>
-    <tableColumn id="3" name="Description"/>
-    <tableColumn id="4" name="Other end"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Pinout2" displayName="Pinout2" ref="A1:D50" headerRowCount="1">
-  <autoFilter ref="A1:D50"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Pin"/>
-    <tableColumn id="2" name="Wire"/>
-    <tableColumn id="3" name="Description"/>
-    <tableColumn id="4" name="Other end"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Pinout3" displayName="Pinout3" ref="A1:D7" headerRowCount="1">
-  <autoFilter ref="A1:D7"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Pin"/>
-    <tableColumn id="2" name="Wire"/>
-    <tableColumn id="3" name="Description"/>
-    <tableColumn id="4" name="Other end"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Pinout4" displayName="Pinout4" ref="A1:D7" headerRowCount="1">
-  <autoFilter ref="A1:D7"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Pin"/>
-    <tableColumn id="2" name="Wire"/>
-    <tableColumn id="3" name="Description"/>
-    <tableColumn id="4" name="Other end"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Pinout5" displayName="Pinout5" ref="A1:D9" headerRowCount="1">
-  <autoFilter ref="A1:D9"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Pin"/>
-    <tableColumn id="2" name="Wire"/>
-    <tableColumn id="3" name="Description"/>
-    <tableColumn id="4" name="Other end"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Pinout6" displayName="Pinout6" ref="A1:D9" headerRowCount="1">
-  <autoFilter ref="A1:D9"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Pin"/>
-    <tableColumn id="2" name="Wire"/>
-    <tableColumn id="3" name="Description"/>
-    <tableColumn id="4" name="Other end"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -578,792 +540,798 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>ECU-A ecu_a</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>Pin</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Wire</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Other end</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>w111_c</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Injector 4 drive (-)</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 34</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>w110_c</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Injector 3 drive (-)</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 33</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>w109_c</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Injector 2 drive (-)</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 32</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>A4</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>w108_c</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Injector 1 drive (-)</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 31</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>A5</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>w78</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>ECU main +12 V</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>splice sp_sw12 (SP-SW12: switched +12 V)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>A6</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>w19</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>+8 V sensor supply</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>splice sp_8v (SP-8V: +8 V cam sensor supply)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>A7</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>w_drain_ecu_a</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Shield drain</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>A8</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>w200_c</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Crank sensor signal</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 9</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>A9</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>w_trig2_pin</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Cam sensor signal</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>splice sp_trig2 (SP-CAM: cam signal + 1.8k pull-up to +8V)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>A10</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>w123_c</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>Coil 4 trigger (IGT)</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 38</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>A11</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>w122_c</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Coil 3 trigger (IGT)</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 37</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>A12</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>w121_c</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>Coil 2 trigger (IGT)</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 36</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>A13</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>w120_c</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Coil 1 trigger (IGT)</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 35</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>A14</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>w38</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>Pedal 1 signal main</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>PEDAL pin 6</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>A15</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>w201_c</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Coolant temp signal</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 40</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>A16</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>w202_c</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>Intake temp signal</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 41</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>A17</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>w26_c</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>MAP sensor signal</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 30</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>A18</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>w_ac_kill</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>A/C cancel (ACT)</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>OEM A/C amplifier pin 11</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>A19</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>w_fp85</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Fuel pump relay (-)</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>FP RELAY K1 pin 85</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>A20</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>w81</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>ETB relay coil (-)</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D22" s="10" t="inlineStr">
         <is>
           <t>LOGIC M4 pin 85</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>A21</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>w103_c</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Boost solenoid (-)</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 39</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>A22</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>w128_c</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>Throttle pos 1 main</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 24</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>A23</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>cab_fspur_l</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>FL conditioned out</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>FRONT WS INLINE pin 3</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>A24</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>w68</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>Sensor ground</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D26" s="10" t="inlineStr">
         <is>
           <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>A25</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>w70</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>ECU power ground</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>splice sp_chassis (SP-GND-CHASSIS: ECU power ground)</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>A26</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>w_str85</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>Start relay coil (-)</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D28" s="10" t="inlineStr">
         <is>
           <t>POWER R3 pin 85</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>A27</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>w_mrs_c</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>EHPS pump speed</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 44</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>A28</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>w76</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>EFI relay coil (-)</t>
         </is>
       </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="D30" s="10" t="inlineStr">
         <is>
           <t>POWER R2 pin 85</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>A29</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>w_fan85</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>Rad fan relay (-)</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>POWER R4 pin 85</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="7" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>A30</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>w16_c</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>Turbo speed signal</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D32" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 17</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>A31</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>w48_c</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>Flex fuel signal</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 21</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="7" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>A32</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>w67</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>+5 V sensor supply</t>
         </is>
       </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="D34" s="10" t="inlineStr">
         <is>
           <t>splice sp_5v (SP-5V-A: +5 V sensor supply)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>A33</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>w129_c</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>Throttle pos 2 sub</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 25</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="7" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>A34</t>
         </is>
       </c>
-      <c r="B35" s="7" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>w_a34</t>
         </is>
       </c>
-      <c r="C35" s="8" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>ECU power ground</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D36" s="10" t="inlineStr">
         <is>
           <t>splice sp_chassis (SP-GND-CHASSIS: ECU power ground)</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A2:D36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1371,960 +1339,966 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>BULKHEAD bh_a_fw</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>Pin</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Wire</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Other end</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="n">
+    <row r="3">
+      <c r="A3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>w_inj_pwr_ac</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Injector +12 V feed</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>FB-LOGIC pin BUS2-4</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="7" t="n">
+    <row r="4">
+      <c r="A4" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>w_cop_pwr_ac</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Coil +12 V feed</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>FB-LOGIC pin BUS2-3</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
+    <row r="5">
+      <c r="A5" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>w200_c</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Crank sensor signal</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A8</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+    <row r="6">
+      <c r="A6" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>w_gnd_a_c41</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Gnd crank sensor</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>SENSOR GND BUS pin 3</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>w_shc_crank</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Crank sensor shield</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+    <row r="8">
+      <c r="A8" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>w_rail_sp_8v_c</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>+8 V to cam sensor</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>splice sp_8v (SP-8V: +8 V cam sensor supply)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
+    <row r="9">
+      <c r="A9" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>w_cam_sig_c</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Cam sensor signal</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>splice sp_trig2 (SP-CAM: cam signal + 1.8k pull-up to +8V)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="n">
+    <row r="10">
+      <c r="A10" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>w_gnd_a_c42</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Gnd cam sensor</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>SENSOR GND BUS pin 4</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
+    <row r="11">
+      <c r="A11" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>w_shc_cam</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Cam sensor shield</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="n">
+    <row r="12">
+      <c r="A12" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>w_5v_a_c40</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>+5 V turbo speed</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>+5V BUS pin 4</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
+    <row r="13">
+      <c r="A13" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>w16_c</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Turbo speed signal</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A30</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="7" t="n">
+    <row r="14">
+      <c r="A14" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>w_gnd_a_c43</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>Gnd turbo speed</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>SENSOR GND BUS pin 5</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="n">
+    <row r="15">
+      <c r="A15" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>w_shc_turbo</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Turbo speed shield</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="n">
+    <row r="16">
+      <c r="A16" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>w_rail_sp_sw12_c</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>+12 V boost + flex</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>splice sp_sw12 (SP-SW12: switched +12 V)</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
+    <row r="17">
+      <c r="A17" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>w48_c</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Flex fuel signal</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A31</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="7" t="n">
+    <row r="18">
+      <c r="A18" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>w_shc_flex</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>Flex fuel shield</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
+    <row r="19">
+      <c r="A19" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>w_rail_sp_5v_c</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>+5 V throttle sensor</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>+5V BUS pin 2</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="7" t="n">
+    <row r="20">
+      <c r="A20" s="8" t="n">
         <v>24</v>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>w128_c</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>Throttle pos 1 main</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>ECU-A pin A22</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
+    <row r="21">
+      <c r="A21" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>w129_c</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Throttle pos 2 sub</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A33</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="7" t="n">
+    <row r="22">
+      <c r="A22" s="8" t="n">
         <v>26</v>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>w_rail_sp_gndout_c</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>Gnd IAT/TPS/coolant</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D22" s="10" t="inlineStr">
         <is>
           <t>SENSOR GND BUS pin 2</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="n">
+    <row r="23">
+      <c r="A23" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>w_shc_etbs</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Throttle shield</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="7" t="n">
+    <row r="24">
+      <c r="A24" s="8" t="n">
         <v>28</v>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>w_5v_a_c39</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>+5 V MAP sensor</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>+5V BUS pin 3</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="n">
+    <row r="25">
+      <c r="A25" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>w_gnd_a_c44</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>Gnd flex + MAP</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>SENSOR GND BUS pin 6</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="7" t="n">
+    <row r="26">
+      <c r="A26" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>w26_c</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>MAP sensor signal</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D26" s="10" t="inlineStr">
         <is>
           <t>ECU-A pin A17</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="n">
+    <row r="27">
+      <c r="A27" s="5" t="n">
         <v>31</v>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>w108_c</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>Injector 1 drive (-)</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A4</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="7" t="n">
+    <row r="28">
+      <c r="A28" s="8" t="n">
         <v>32</v>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>w109_c</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>Injector 2 drive (-)</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D28" s="10" t="inlineStr">
         <is>
           <t>ECU-A pin A3</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="n">
+    <row r="29">
+      <c r="A29" s="5" t="n">
         <v>33</v>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>w110_c</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>Injector 3 drive (-)</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A2</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="7" t="n">
+    <row r="30">
+      <c r="A30" s="8" t="n">
         <v>34</v>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>w111_c</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>Injector 4 drive (-)</t>
         </is>
       </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="D30" s="10" t="inlineStr">
         <is>
           <t>ECU-A pin A1</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="n">
+    <row r="31">
+      <c r="A31" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>w120_c</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>Coil 1 trigger (IGT)</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A13</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="7" t="n">
+    <row r="32">
+      <c r="A32" s="8" t="n">
         <v>36</v>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>w121_c</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>Coil 2 trigger (IGT)</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D32" s="10" t="inlineStr">
         <is>
           <t>ECU-A pin A12</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="n">
+    <row r="33">
+      <c r="A33" s="5" t="n">
         <v>37</v>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>w122_c</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>Coil 3 trigger (IGT)</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A11</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="7" t="n">
+    <row r="34">
+      <c r="A34" s="8" t="n">
         <v>38</v>
       </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>w123_c</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>Coil 4 trigger (IGT)</t>
         </is>
       </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="D34" s="10" t="inlineStr">
         <is>
           <t>ECU-A pin A10</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="n">
+    <row r="35">
+      <c r="A35" s="5" t="n">
         <v>39</v>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>w103_c</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>Boost solenoid (-)</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A21</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="7" t="n">
+    <row r="36">
+      <c r="A36" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="B35" s="7" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>w201_c</t>
         </is>
       </c>
-      <c r="C35" s="8" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>Coolant temp signal</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D36" s="10" t="inlineStr">
         <is>
           <t>ECU-A pin A15</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="n">
+    <row r="37">
+      <c r="A37" s="5" t="n">
         <v>41</v>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>w202_c</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>Intake temp signal</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A16</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="7" t="n">
+    <row r="38">
+      <c r="A38" s="8" t="n">
         <v>42</v>
       </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t>w_fb_mrs_en</t>
         </is>
       </c>
-      <c r="C37" s="8" t="inlineStr">
+      <c r="C38" s="9" t="inlineStr">
         <is>
           <t>EHPS enable +12 V</t>
         </is>
       </c>
-      <c r="D37" s="9" t="inlineStr">
+      <c r="D38" s="10" t="inlineStr">
         <is>
           <t>FB-LOGIC pin BUS2-12</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="n">
+    <row r="39">
+      <c r="A39" s="5" t="n">
         <v>44</v>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>w_mrs_c</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>EHPS pump speed</t>
         </is>
       </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="D39" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A27</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="7" t="n">
+    <row r="40">
+      <c r="A40" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="B39" s="7" t="inlineStr"/>
-      <c r="C39" s="8" t="inlineStr">
+      <c r="B40" s="8" t="inlineStr"/>
+      <c r="C40" s="9" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D39" s="9" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="n">
+      <c r="D40" s="10" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="B40" s="4" t="inlineStr"/>
-      <c r="C40" s="5" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr"/>
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="7" t="n">
+      <c r="D41" s="7" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n">
         <v>47</v>
       </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="B42" s="8" t="inlineStr">
         <is>
           <t>w_5v_brail_c45</t>
         </is>
       </c>
-      <c r="C41" s="8" t="inlineStr">
+      <c r="C42" s="9" t="inlineStr">
         <is>
           <t>+5 V oil pressure</t>
         </is>
       </c>
-      <c r="D41" s="9" t="inlineStr">
+      <c r="D42" s="10" t="inlineStr">
         <is>
           <t>+5V BUS pin 5</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="4" t="n">
+    <row r="43">
+      <c r="A43" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="B42" s="4" t="inlineStr">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>w_5v_brail_c46</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>+5 V fuel pressure</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="D43" s="7" t="inlineStr">
         <is>
           <t>+5V BUS pin 6</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="7" t="n">
+    <row r="44">
+      <c r="A44" s="8" t="n">
         <v>51</v>
       </c>
-      <c r="B43" s="7" t="inlineStr">
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>w_5v_brail_c47</t>
         </is>
       </c>
-      <c r="C43" s="8" t="inlineStr">
+      <c r="C44" s="9" t="inlineStr">
         <is>
           <t>+5 V coolant press</t>
         </is>
       </c>
-      <c r="D43" s="9" t="inlineStr">
+      <c r="D44" s="10" t="inlineStr">
         <is>
           <t>+5V BUS pin 7</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="n">
+    <row r="45">
+      <c r="A45" s="5" t="n">
         <v>52</v>
       </c>
-      <c r="B44" s="4" t="inlineStr"/>
-      <c r="C44" s="5" t="inlineStr">
+      <c r="B45" s="5" t="inlineStr"/>
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D44" s="6" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="7" t="n">
+      <c r="D45" s="7" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="n">
         <v>53</v>
       </c>
-      <c r="B45" s="7" t="inlineStr"/>
-      <c r="C45" s="8" t="inlineStr">
+      <c r="B46" s="8" t="inlineStr"/>
+      <c r="C46" s="9" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D45" s="9" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="n">
+      <c r="D46" s="10" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="n">
         <v>56</v>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>w_eps_rly</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>EHPS relay coil (-)</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr">
+      <c r="D47" s="7" t="inlineStr">
         <is>
           <t>EHPS RELAY pin 85</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="7" t="n">
+    <row r="48">
+      <c r="A48" s="8" t="n">
         <v>57</v>
       </c>
-      <c r="B47" s="7" t="inlineStr"/>
-      <c r="C47" s="8" t="inlineStr">
+      <c r="B48" s="8" t="inlineStr"/>
+      <c r="C48" s="9" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D47" s="9" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="n">
+      <c r="D48" s="10" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="n">
         <v>58</v>
       </c>
-      <c r="B48" s="4" t="inlineStr"/>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr"/>
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D48" s="6" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="7" t="n">
+      <c r="D49" s="7" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="n">
         <v>59</v>
       </c>
-      <c r="B49" s="7" t="inlineStr"/>
-      <c r="C49" s="8" t="inlineStr">
+      <c r="B50" s="8" t="inlineStr"/>
+      <c r="C50" s="9" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D49" s="9" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="n">
+      <c r="D50" s="10" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="n">
         <v>61</v>
       </c>
-      <c r="B50" s="4" t="inlineStr"/>
-      <c r="C50" s="5" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr"/>
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D50" s="6" t="inlineStr"/>
+      <c r="D51" s="7" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A2:D51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2332,156 +2306,162 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>FRONT WS INLINE ix_ws_front_p</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>Pin</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Wire</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Other end</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="n">
+    <row r="3">
+      <c r="A3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>cab_fspur_5v</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>VRC-F +5V</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>splice sp_5v (SP-5V-A: +5 V sensor supply)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="7" t="n">
+    <row r="4">
+      <c r="A4" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>cab_fspur_gnd</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>VRC-F GND</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
+    <row r="5">
+      <c r="A5" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>cab_fspur_l</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>FL conditioned out</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>ECU-A pin A23</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+    <row r="6">
+      <c r="A6" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>cab_fspur_r_ac</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>FR conditioned out</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>ECU-B (Link G4X plug B, centre dash) pin B21</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>cab_fspur_sh</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>WS-F screen drain</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+    <row r="8">
+      <c r="A8" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr"/>
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr"/>
+      <c r="D8" s="10" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A2:D8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2489,164 +2469,170 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>PEDAL aps</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>Pin</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Wire</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Other end</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="n">
+    <row r="3">
+      <c r="A3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>w210</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>+5 V pedal sensor 2</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>splice sp_5v_2 (SP-5V-PEDAL: +5 V to pedal + cruise)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="7" t="n">
+    <row r="4">
+      <c r="A4" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>w_aps_gnd2</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Pedal 2 ground</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
+    <row r="5">
+      <c r="A5" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>w_aps_vpa2</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Pedal 2 signal sub</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>ECU-B (Link G4X plug B, centre dash) pin B33</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+    <row r="6">
+      <c r="A6" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>w_aps_vc1</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>+5 V pedal sensor 1</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>splice sp_5v_2 (SP-5V-PEDAL: +5 V to pedal + cruise)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>w40</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Pedal 1 ground</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+    <row r="8">
+      <c r="A8" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>w38</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Pedal 1 signal main</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>ECU-A pin A14</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A2:D8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2654,196 +2640,202 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>+5V BUS bus_5v_bha_p</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>Pin</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Wire</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Other end</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="n">
+    <row r="3">
+      <c r="A3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>w_5v_bha_trunk</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>+5 V sensor supply</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>splice sp_5v (SP-5V-A: +5 V sensor supply)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="7" t="n">
+    <row r="4">
+      <c r="A4" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>w_rail_sp_5v_c</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>+5 V throttle sensor</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 23</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
+    <row r="5">
+      <c r="A5" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>w_5v_a_c39</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>+5 V MAP sensor</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 28</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+    <row r="6">
+      <c r="A6" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>w_5v_a_c40</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>+5 V turbo speed</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 16</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>w_5v_brail_c45</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>+5 V oil pressure</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 47</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+    <row r="8">
+      <c r="A8" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>w_5v_brail_c46</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>+5 V fuel pressure</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 50</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
+    <row r="9">
+      <c r="A9" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>w_5v_brail_c47</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>+5 V coolant press</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 51</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="n">
+    <row r="10">
+      <c r="A10" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="inlineStr"/>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr"/>
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr"/>
+      <c r="D10" s="10" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A2:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2851,187 +2843,193 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>SENSOR GND BUS bus_gnd_bha_p</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>Pin</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Wire</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Other end</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="n">
+    <row r="3">
+      <c r="A3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>w_gnd_bha_trunk</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Sensor ground</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>splice sp_gndout (SP-GNDOUT-A: sensor ground)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="7" t="n">
+    <row r="4">
+      <c r="A4" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>w_rail_sp_gndout_c</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Gnd IAT/TPS/coolant</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 26</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
+    <row r="5">
+      <c r="A5" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>w_gnd_a_c41</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Gnd crank sensor</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 10</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+    <row r="6">
+      <c r="A6" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>w_gnd_a_c42</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Gnd cam sensor</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 14</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>w_gnd_a_c43</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Gnd turbo speed</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>BULKHEAD pin 18</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+    <row r="8">
+      <c r="A8" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>w_gnd_a_c44</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Gnd flex + MAP</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>BULKHEAD pin 29</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
+    <row r="9">
+      <c r="A9" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="inlineStr"/>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr"/>
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="n">
+      <c r="D9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="inlineStr"/>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr"/>
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr"/>
+      <c r="D10" s="10" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A2:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
wirelist xlsx: match Dan's styled reference (group-title row, grouped column order, reference palette, freeze C3, per-connector pinout sheets); CSV order unchanged
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/A-cabin-pinouts.xlsx
+++ b/docs/harness/wirelist/A-cabin-pinouts.xlsx
@@ -7,26 +7,26 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ECU-A ecu_a" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="BULKHEAD bh_a_fw" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="FRONT WS INLINE ix_ws_front_p" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="PEDAL aps" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="+5V BUS bus_5v_bha_p" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="SENSOR GND BUS bus_gnd_bha_p" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ECU-A (ecu_a)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="BULKHEAD (bh_a_fw)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="FRONT WS INLINE (ix_ws_front_p)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="PEDAL (aps)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="+5V BUS (bus_5v_bha_p)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="SENSOR GND BUS (bus_gnd_bha_p)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ECU-A ecu_a'!$A$2:$D$36</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'ECU-A ecu_a'!$2:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BULKHEAD bh_a_fw'!$A$2:$D$51</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'BULKHEAD bh_a_fw'!$2:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'FRONT WS INLINE ix_ws_front_p'!$A$2:$D$8</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'FRONT WS INLINE ix_ws_front_p'!$2:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PEDAL aps'!$A$2:$D$8</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'PEDAL aps'!$2:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'+5V BUS bus_5v_bha_p'!$A$2:$D$10</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'+5V BUS bus_5v_bha_p'!$2:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'SENSOR GND BUS bus_gnd_bha_p'!$A$2:$D$10</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'SENSOR GND BUS bus_gnd_bha_p'!$2:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ECU-A (ecu_a)'!$A$2:$D$36</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'ECU-A (ecu_a)'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BULKHEAD (bh_a_fw)'!$A$2:$D$51</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'BULKHEAD (bh_a_fw)'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'FRONT WS INLINE (ix_ws_front_p)'!$A$2:$D$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'FRONT WS INLINE (ix_ws_front_p)'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PEDAL (aps)'!$A$2:$D$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'PEDAL (aps)'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'+5V BUS (bus_5v_bha_p)'!$A$2:$D$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'+5V BUS (bus_5v_bha_p)'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'SENSOR GND BUS (bus_gnd_bha_p)'!$A$2:$D$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'SENSOR GND BUS (bus_gnd_bha_p)'!$1:$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -49,14 +49,13 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F1F1F"/>
       <sz val="12"/>
     </font>
     <font>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -65,47 +64,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BFBFBF"/>
+        <fgColor rgb="00E7E6F7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDEDED"/>
+        <fgColor rgb="00F3F2FB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8F8F8"/>
+        <fgColor rgb="00C9DDF5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="009DC3E6"/>
+        <fgColor rgb="00E4EEFA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
+        <fgColor rgb="00CDEBCB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EEF5FB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00A9D18E"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2F0D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F1F8EC"/>
+        <fgColor rgb="00E6F5E5"/>
       </patternFill>
     </fill>
   </fills>
@@ -153,28 +137,28 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -554,7 +538,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ECU-A ecu_a</t>
+          <t>ECU-A (ecu_a)</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1337,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BULKHEAD bh_a_fw</t>
+          <t>BULKHEAD (bh_a_fw)</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2304,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FRONT WS INLINE ix_ws_front_p</t>
+          <t>FRONT WS INLINE (ix_ws_front_p)</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2467,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PEDAL aps</t>
+          <t>PEDAL (aps)</t>
         </is>
       </c>
     </row>
@@ -2654,7 +2638,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>+5V BUS bus_5v_bha_p</t>
+          <t>+5V BUS (bus_5v_bha_p)</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2841,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SENSOR GND BUS bus_gnd_bha_p</t>
+          <t>SENSOR GND BUS (bus_gnd_bha_p)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
wirelist xlsx: match Dan's styled reference (group-title row, grouped column order, reference palette, freeze C3, per-connector pinout sheets); CSV order unchanged (#338)
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/A-cabin-pinouts.xlsx
+++ b/docs/harness/wirelist/A-cabin-pinouts.xlsx
@@ -7,26 +7,26 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ECU-A ecu_a" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="BULKHEAD bh_a_fw" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="FRONT WS INLINE ix_ws_front_p" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="PEDAL aps" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="+5V BUS bus_5v_bha_p" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="SENSOR GND BUS bus_gnd_bha_p" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ECU-A (ecu_a)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="BULKHEAD (bh_a_fw)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="FRONT WS INLINE (ix_ws_front_p)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="PEDAL (aps)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="+5V BUS (bus_5v_bha_p)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="SENSOR GND BUS (bus_gnd_bha_p)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ECU-A ecu_a'!$A$2:$D$36</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'ECU-A ecu_a'!$2:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BULKHEAD bh_a_fw'!$A$2:$D$51</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'BULKHEAD bh_a_fw'!$2:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'FRONT WS INLINE ix_ws_front_p'!$A$2:$D$8</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'FRONT WS INLINE ix_ws_front_p'!$2:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PEDAL aps'!$A$2:$D$8</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'PEDAL aps'!$2:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'+5V BUS bus_5v_bha_p'!$A$2:$D$10</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'+5V BUS bus_5v_bha_p'!$2:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'SENSOR GND BUS bus_gnd_bha_p'!$A$2:$D$10</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'SENSOR GND BUS bus_gnd_bha_p'!$2:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ECU-A (ecu_a)'!$A$2:$D$36</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'ECU-A (ecu_a)'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BULKHEAD (bh_a_fw)'!$A$2:$D$51</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'BULKHEAD (bh_a_fw)'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'FRONT WS INLINE (ix_ws_front_p)'!$A$2:$D$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'FRONT WS INLINE (ix_ws_front_p)'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PEDAL (aps)'!$A$2:$D$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'PEDAL (aps)'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'+5V BUS (bus_5v_bha_p)'!$A$2:$D$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'+5V BUS (bus_5v_bha_p)'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'SENSOR GND BUS (bus_gnd_bha_p)'!$A$2:$D$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'SENSOR GND BUS (bus_gnd_bha_p)'!$1:$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -49,14 +49,13 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F1F1F"/>
       <sz val="12"/>
     </font>
     <font>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -65,47 +64,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BFBFBF"/>
+        <fgColor rgb="00E7E6F7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDEDED"/>
+        <fgColor rgb="00F3F2FB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8F8F8"/>
+        <fgColor rgb="00C9DDF5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="009DC3E6"/>
+        <fgColor rgb="00E4EEFA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
+        <fgColor rgb="00CDEBCB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EEF5FB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00A9D18E"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2F0D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F1F8EC"/>
+        <fgColor rgb="00E6F5E5"/>
       </patternFill>
     </fill>
   </fills>
@@ -153,28 +137,28 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -554,7 +538,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ECU-A ecu_a</t>
+          <t>ECU-A (ecu_a)</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1337,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BULKHEAD bh_a_fw</t>
+          <t>BULKHEAD (bh_a_fw)</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2304,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FRONT WS INLINE ix_ws_front_p</t>
+          <t>FRONT WS INLINE (ix_ws_front_p)</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2467,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PEDAL aps</t>
+          <t>PEDAL (aps)</t>
         </is>
       </c>
     </row>
@@ -2654,7 +2638,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>+5V BUS bus_5v_bha_p</t>
+          <t>+5V BUS (bus_5v_bha_p)</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2841,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SENSOR GND BUS bus_gnd_bha_p</t>
+          <t>SENSOR GND BUS (bus_gnd_bha_p)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SoT switch: wire lists become the wiring SoT; apply gap answers (R206)
- IG2 -> 1N5822 diode -> A5 wake feed on A-cabin (sp_a5, d_ig2_wake, circuit IG2WAKE)
- comms pin C1 set nc; GNDOUT -> GNDOUT_A / GNDOUT_B; A5 = SW12
- flex pin letters, opto board pin names; drawing-only splice/end names are now SoT
- wirelist.py --check: channels.csv vs lists both ways, hard for every list
- DECISIONS R206 added; R18, R78, R108, R144, R146 removed, CAD comments repointed
- OPEN-ITEMS: N45/N46 -> N48/N49 closed, N38 filled, row 145 (EWD pages)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/A-cabin-pinouts.xlsx
+++ b/docs/harness/wirelist/A-cabin-pinouts.xlsx
@@ -660,7 +660,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>w78</t>
+          <t>w_a5_pin</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>splice sp_sw12 (SP-SW12: switched +12 V)</t>
+          <t>splice sp_a5 (SP-A5: ECU main feed, SW12 + IG2 diode)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SoT switch: wire lists become the wiring SoT; apply gap answers (R206) (#341)
- IG2 -> 1N5822 diode -> A5 wake feed on A-cabin (sp_a5, d_ig2_wake, circuit IG2WAKE)
- comms pin C1 set nc; GNDOUT -> GNDOUT_A / GNDOUT_B; A5 = SW12
- flex pin letters, opto board pin names; drawing-only splice/end names are now SoT
- wirelist.py --check: channels.csv vs lists both ways, hard for every list
- DECISIONS R206 added; R18, R78, R108, R144, R146 removed, CAD comments repointed
- OPEN-ITEMS: N45/N46 -> N48/N49 closed, N38 filled, row 145 (EWD pages)

Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/A-cabin-pinouts.xlsx
+++ b/docs/harness/wirelist/A-cabin-pinouts.xlsx
@@ -660,7 +660,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>w78</t>
+          <t>w_a5_pin</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>splice sp_sw12 (SP-SW12: switched +12 V)</t>
+          <t>splice sp_a5 (SP-A5: ECU main feed, SW12 + IG2 diode)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DRB102 bulkhead reassigned by device (R208); the cavity map is generated
- bulkhead_assign.py: each engine/cabin circuit is one wire, grouped by device in route order, cut into contiguous cavity runs; same cavity both halves; no A/B sections (loom ownership stays on the connector id)
- every cavity id is c<DRB number>; lists, four bulkhead drawings, map, labels and test_gates updated
- gauge / contact size / rating limits checked (audit_cavity_parts, audit_mating M8, script limits)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/A-cabin-pinouts.xlsx
+++ b/docs/harness/wirelist/A-cabin-pinouts.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ECU-A (ecu_a)'!$A$2:$D$36</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'ECU-A (ecu_a)'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BULKHEAD (bh_a_fw)'!$A$2:$D$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BULKHEAD (bh_a_fw)'!$A$2:$D$71</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'BULKHEAD (bh_a_fw)'!$1:$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'FRONT WS INLINE (ix_ws_front_p)'!$A$2:$D$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'FRONT WS INLINE (ix_ws_front_p)'!$1:$2</definedName>
@@ -582,7 +582,7 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 34</t>
+          <t>BULKHEAD pin 24</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 33</t>
+          <t>BULKHEAD pin 23</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 32</t>
+          <t>BULKHEAD pin 22</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 31</t>
+          <t>BULKHEAD pin 21</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 9</t>
+          <t>BULKHEAD pin 74</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 38</t>
+          <t>BULKHEAD pin 12</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 37</t>
+          <t>BULKHEAD pin 11</t>
         </is>
       </c>
     </row>
@@ -824,7 +824,7 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 36</t>
+          <t>BULKHEAD pin 10</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 35</t>
+          <t>BULKHEAD pin 9</t>
         </is>
       </c>
     </row>
@@ -890,7 +890,7 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 40</t>
+          <t>BULKHEAD pin 70</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 41</t>
+          <t>BULKHEAD pin 33</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 30</t>
+          <t>BULKHEAD pin 17</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 39</t>
+          <t>BULKHEAD pin 58</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 24</t>
+          <t>BULKHEAD pin 42</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 44</t>
+          <t>BULKHEAD pin 84</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 17</t>
+          <t>BULKHEAD pin 53</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 21</t>
+          <t>BULKHEAD pin 31</t>
         </is>
       </c>
     </row>
@@ -1286,7 +1286,7 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 25</t>
+          <t>BULKHEAD pin 44</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1369,17 +1369,17 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>w_inj_pwr_ac</t>
+          <t>w_cop_pwr_ac</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Injector +12 V feed</t>
+          <t>Coil +12 V feed</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>FB-LOGIC pin BUS2-4</t>
+          <t>FB-LOGIC pin BUS2-3</t>
         </is>
       </c>
     </row>
@@ -1389,723 +1389,611 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>w_cop_pwr_ac</t>
+          <t>w_inj_pwr_ac</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Coil +12 V feed</t>
+          <t>Injector +12 V feed</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>FB-LOGIC pin BUS2-3</t>
+          <t>FB-LOGIC pin BUS2-4</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>w200_c</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr"/>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Crank sensor signal</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>ECU-A pin A8</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>w_gnd_a_c41</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr"/>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Gnd crank sensor</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>SENSOR GND BUS pin 3</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>w_shc_crank</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr"/>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Crank sensor shield</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>w_rail_sp_8v_c</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr"/>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>+8 V to cam sensor</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>splice sp_8v (SP-8V: +8 V cam sensor supply)</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>w_cam_sig_c</t>
-        </is>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr"/>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Cam sensor signal</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>splice sp_trig2 (SP-CAM: cam signal + 1.8k pull-up to +8V)</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
-        <v>14</v>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>w_gnd_a_c42</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr"/>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Gnd cam sensor</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>SENSOR GND BUS pin 4</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>w_shc_cam</t>
+          <t>w120_c</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Cam sensor shield</t>
+          <t>Coil 1 trigger (IGT)</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>ECU-A pin A13</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>w_5v_a_c40</t>
+          <t>w121_c</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>+5 V turbo speed</t>
+          <t>Coil 2 trigger (IGT)</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>+5V BUS pin 4</t>
+          <t>ECU-A pin A12</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>w16_c</t>
+          <t>w122_c</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Turbo speed signal</t>
+          <t>Coil 3 trigger (IGT)</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>ECU-A pin A30</t>
+          <t>ECU-A pin A11</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>w_gnd_a_c43</t>
+          <t>w123_c</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Gnd turbo speed</t>
+          <t>Coil 4 trigger (IGT)</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>SENSOR GND BUS pin 5</t>
+          <t>ECU-A pin A10</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>w_shc_turbo</t>
+          <t>w_5v_brail_c46</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Turbo speed shield</t>
+          <t>+5 V fuel pressure</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>+5V BUS pin 6</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>w_rail_sp_sw12_c</t>
+          <t>w_5v_a_c39</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>+12 V boost + flex</t>
+          <t>+5 V MAP sensor</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>splice sp_sw12 (SP-SW12: switched +12 V)</t>
+          <t>+5V BUS pin 3</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>w48_c</t>
+          <t>w26_c</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Flex fuel signal</t>
+          <t>MAP sensor signal</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>ECU-A pin A31</t>
+          <t>ECU-A pin A17</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>w_shc_flex</t>
+          <t>w_gnd_a_c44</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Flex fuel shield</t>
+          <t>Gnd flex + MAP</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>SENSOR GND BUS pin 6</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>23</v>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>w_rail_sp_5v_c</t>
-        </is>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr"/>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>+5 V throttle sensor</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>+5V BUS pin 2</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n">
-        <v>24</v>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>w128_c</t>
-        </is>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="B20" s="8" t="inlineStr"/>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Throttle pos 1 main</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>ECU-A pin A22</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>w129_c</t>
+          <t>w108_c</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Throttle pos 2 sub</t>
+          <t>Injector 1 drive (-)</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>ECU-A pin A33</t>
+          <t>ECU-A pin A4</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>w_rail_sp_gndout_c</t>
+          <t>w109_c</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Gnd IAT/TPS/coolant</t>
+          <t>Injector 2 drive (-)</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>SENSOR GND BUS pin 2</t>
+          <t>ECU-A pin A3</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>w_shc_etbs</t>
+          <t>w110_c</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Throttle shield</t>
+          <t>Injector 3 drive (-)</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>ECU-A pin A2</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>w_5v_a_c39</t>
+          <t>w111_c</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>+5 V MAP sensor</t>
+          <t>Injector 4 drive (-)</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>+5V BUS pin 3</t>
+          <t>ECU-A pin A1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>w_gnd_a_c44</t>
+          <t>w_5v_brail_c47</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Gnd flex + MAP</t>
+          <t>+5 V coolant press</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>SENSOR GND BUS pin 6</t>
+          <t>+5V BUS pin 7</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>w26_c</t>
+          <t>w_5v_brail_c45</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>MAP sensor signal</t>
+          <t>+5 V oil pressure</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>ECU-A pin A17</t>
+          <t>+5V BUS pin 5</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>w108_c</t>
+          <t>w_rail_sp_sw12_c</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Injector 1 drive (-)</t>
+          <t>+12 V boost + flex</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>ECU-A pin A4</t>
+          <t>splice sp_sw12 (SP-SW12: switched +12 V)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>w109_c</t>
+          <t>w48_c</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Injector 2 drive (-)</t>
+          <t>Flex fuel signal</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>ECU-A pin A3</t>
+          <t>ECU-A pin A31</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>w110_c</t>
+          <t>w_shc_flex</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Injector 3 drive (-)</t>
+          <t>Flex fuel shield</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>ECU-A pin A2</t>
+          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>w111_c</t>
+          <t>w202_c</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>Injector 4 drive (-)</t>
+          <t>Intake temp signal</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>ECU-A pin A1</t>
+          <t>ECU-A pin A16</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>w120_c</t>
+          <t>w_rail_sp_gndout_c</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Coil 1 trigger (IGT)</t>
+          <t>Gnd IAT/TPS/coolant</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>ECU-A pin A13</t>
+          <t>SENSOR GND BUS pin 2</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="n">
-        <v>36</v>
-      </c>
-      <c r="B32" s="8" t="inlineStr">
-        <is>
-          <t>w121_c</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="B32" s="8" t="inlineStr"/>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Coil 2 trigger (IGT)</t>
-        </is>
-      </c>
-      <c r="D32" s="10" t="inlineStr">
-        <is>
-          <t>ECU-A pin A12</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n">
-        <v>37</v>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>w122_c</t>
-        </is>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="B33" s="5" t="inlineStr"/>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Coil 3 trigger (IGT)</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>ECU-A pin A11</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="n">
-        <v>38</v>
-      </c>
-      <c r="B34" s="8" t="inlineStr">
-        <is>
-          <t>w123_c</t>
-        </is>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="B34" s="8" t="inlineStr"/>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>Coil 4 trigger (IGT)</t>
-        </is>
-      </c>
-      <c r="D34" s="10" t="inlineStr">
-        <is>
-          <t>ECU-A pin A10</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
-        <v>39</v>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>w103_c</t>
-        </is>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="B35" s="5" t="inlineStr"/>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Boost solenoid (-)</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>ECU-A pin A21</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>w201_c</t>
-        </is>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="B36" s="8" t="inlineStr"/>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>Coolant temp signal</t>
-        </is>
-      </c>
-      <c r="D36" s="10" t="inlineStr">
-        <is>
-          <t>ECU-A pin A15</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n">
-        <v>41</v>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>w202_c</t>
-        </is>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="B37" s="5" t="inlineStr"/>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Intake temp signal</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>ECU-A pin A16</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>w_fb_mrs_en</t>
+          <t>w_rail_sp_5v_c</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>EHPS enable +12 V</t>
+          <t>+5 V throttle sensor</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>FB-LOGIC pin BUS2-12</t>
+          <t>+5V BUS pin 2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>w_mrs_c</t>
+          <t>w128_c</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>EHPS pump speed</t>
+          <t>Throttle pos 1 main</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>ECU-A pin A27</t>
+          <t>ECU-A pin A22</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B40" s="8" t="inlineStr"/>
       <c r="C40" s="9" t="inlineStr">
@@ -2117,15 +2005,23 @@
     </row>
     <row r="41">
       <c r="A41" s="5" t="n">
-        <v>46</v>
-      </c>
-      <c r="B41" s="5" t="inlineStr"/>
+        <v>44</v>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>w129_c</t>
+        </is>
+      </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>spare, sealing plug</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr"/>
+          <t>Throttle pos 2 sub</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>ECU-A pin A33</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="n">
@@ -2133,107 +2029,99 @@
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>w_5v_brail_c45</t>
+          <t>w_shc_etbs</t>
         </is>
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>+5 V oil pressure</t>
+          <t>Throttle shield</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>+5V BUS pin 5</t>
+          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n">
-        <v>50</v>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>w_5v_brail_c46</t>
-        </is>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr"/>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>+5 V fuel pressure</t>
-        </is>
-      </c>
-      <c r="D43" s="7" t="inlineStr">
-        <is>
-          <t>+5V BUS pin 6</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="8" t="n">
-        <v>51</v>
-      </c>
-      <c r="B44" s="8" t="inlineStr">
-        <is>
-          <t>w_5v_brail_c47</t>
-        </is>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="B44" s="8" t="inlineStr"/>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>+5 V coolant press</t>
-        </is>
-      </c>
-      <c r="D44" s="10" t="inlineStr">
-        <is>
-          <t>+5V BUS pin 7</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n">
         <v>52</v>
       </c>
-      <c r="B45" s="5" t="inlineStr"/>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>w_5v_a_c40</t>
+        </is>
+      </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>spare, sealing plug</t>
-        </is>
-      </c>
-      <c r="D45" s="7" t="inlineStr"/>
+          <t>+5 V turbo speed</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>+5V BUS pin 4</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="n">
         <v>53</v>
       </c>
-      <c r="B46" s="8" t="inlineStr"/>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>w16_c</t>
+        </is>
+      </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>spare, sealing plug</t>
-        </is>
-      </c>
-      <c r="D46" s="10" t="inlineStr"/>
+          <t>Turbo speed signal</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>ECU-A pin A30</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n">
-        <v>56</v>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>w_eps_rly</t>
-        </is>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr"/>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>EHPS relay coil (-)</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>EHPS RELAY pin 85</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B48" s="8" t="inlineStr"/>
       <c r="C48" s="9" t="inlineStr">
@@ -2245,42 +2133,394 @@
     </row>
     <row r="49">
       <c r="A49" s="5" t="n">
-        <v>58</v>
-      </c>
-      <c r="B49" s="5" t="inlineStr"/>
+        <v>56</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>w_gnd_a_c43</t>
+        </is>
+      </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>spare, sealing plug</t>
-        </is>
-      </c>
-      <c r="D49" s="7" t="inlineStr"/>
+          <t>Gnd turbo speed</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>SENSOR GND BUS pin 5</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="n">
-        <v>59</v>
-      </c>
-      <c r="B50" s="8" t="inlineStr"/>
+        <v>57</v>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>w_shc_turbo</t>
+        </is>
+      </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>spare, sealing plug</t>
-        </is>
-      </c>
-      <c r="D50" s="10" t="inlineStr"/>
+          <t>Turbo speed shield</t>
+        </is>
+      </c>
+      <c r="D50" s="10" t="inlineStr">
+        <is>
+          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n">
-        <v>61</v>
-      </c>
-      <c r="B51" s="5" t="inlineStr"/>
+        <v>58</v>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>w103_c</t>
+        </is>
+      </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
+          <t>Boost solenoid (-)</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>ECU-A pin A21</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="n">
+        <v>63</v>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>w_rail_sp_8v_c</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>+8 V to cam sensor</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>splice sp_8v (SP-8V: +8 V cam sensor supply)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>w_cam_sig_c</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Cam sensor signal</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>splice sp_trig2 (SP-CAM: cam signal + 1.8k pull-up to +8V)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>w_gnd_a_c42</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>Gnd cam sensor</t>
+        </is>
+      </c>
+      <c r="D54" s="10" t="inlineStr">
+        <is>
+          <t>SENSOR GND BUS pin 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>w_shc_cam</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Cam sensor shield</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>w201_c</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>Coolant temp signal</t>
+        </is>
+      </c>
+      <c r="D56" s="10" t="inlineStr">
+        <is>
+          <t>ECU-A pin A15</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>w200_c</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Crank sensor signal</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>ECU-A pin A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="n">
+        <v>75</v>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>w_gnd_a_c41</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
+        <is>
+          <t>Gnd crank sensor</t>
+        </is>
+      </c>
+      <c r="D58" s="10" t="inlineStr">
+        <is>
+          <t>SENSOR GND BUS pin 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>w_shc_crank</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>Crank sensor shield</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>w_fb_mrs_en</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>EHPS enable +12 V</t>
+        </is>
+      </c>
+      <c r="D60" s="10" t="inlineStr">
+        <is>
+          <t>FB-LOGIC pin BUS2-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="n">
+        <v>84</v>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>w_mrs_c</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>EHPS pump speed</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>ECU-A pin A27</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>w_eps_rly</t>
+        </is>
+      </c>
+      <c r="C62" s="9" t="inlineStr">
+        <is>
+          <t>EHPS relay coil (-)</t>
+        </is>
+      </c>
+      <c r="D62" s="10" t="inlineStr">
+        <is>
+          <t>EHPS RELAY pin 85</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="n">
+        <v>86</v>
+      </c>
+      <c r="B63" s="5" t="inlineStr"/>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D51" s="7" t="inlineStr"/>
+      <c r="D63" s="7" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="B64" s="8" t="inlineStr"/>
+      <c r="C64" s="9" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D64" s="10" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="n">
+        <v>88</v>
+      </c>
+      <c r="B65" s="5" t="inlineStr"/>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="B66" s="8" t="inlineStr"/>
+      <c r="C66" s="9" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D66" s="10" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="B67" s="5" t="inlineStr"/>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="B68" s="8" t="inlineStr"/>
+      <c r="C68" s="9" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D68" s="10" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="n">
+        <v>92</v>
+      </c>
+      <c r="B69" s="5" t="inlineStr"/>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="B70" s="8" t="inlineStr"/>
+      <c r="C70" s="9" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D70" s="10" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="n">
+        <v>94</v>
+      </c>
+      <c r="B71" s="5" t="inlineStr"/>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:D51"/>
+  <autoFilter ref="A2:D71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -2700,7 +2940,7 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 23</t>
+          <t>BULKHEAD pin 41</t>
         </is>
       </c>
     </row>
@@ -2720,7 +2960,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 28</t>
+          <t>BULKHEAD pin 16</t>
         </is>
       </c>
     </row>
@@ -2740,7 +2980,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 16</t>
+          <t>BULKHEAD pin 52</t>
         </is>
       </c>
     </row>
@@ -2760,7 +3000,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 47</t>
+          <t>BULKHEAD pin 27</t>
         </is>
       </c>
     </row>
@@ -2780,7 +3020,7 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 50</t>
+          <t>BULKHEAD pin 13</t>
         </is>
       </c>
     </row>
@@ -2800,7 +3040,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 51</t>
+          <t>BULKHEAD pin 25</t>
         </is>
       </c>
     </row>
@@ -2903,7 +3143,7 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 26</t>
+          <t>BULKHEAD pin 34</t>
         </is>
       </c>
     </row>
@@ -2923,7 +3163,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 10</t>
+          <t>BULKHEAD pin 75</t>
         </is>
       </c>
     </row>
@@ -2943,7 +3183,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 14</t>
+          <t>BULKHEAD pin 65</t>
         </is>
       </c>
     </row>
@@ -2963,7 +3203,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 18</t>
+          <t>BULKHEAD pin 56</t>
         </is>
       </c>
     </row>
@@ -2983,7 +3223,7 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 29</t>
+          <t>BULKHEAD pin 18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DRB102 bulkhead reassigned by device (R208); the cavity map is generated (#348)
- bulkhead_assign.py: each engine/cabin circuit is one wire, grouped by device in route order, cut into contiguous cavity runs; same cavity both halves; no A/B sections (loom ownership stays on the connector id)
- every cavity id is c<DRB number>; lists, four bulkhead drawings, map, labels and test_gates updated
- gauge / contact size / rating limits checked (audit_cavity_parts, audit_mating M8, script limits)

Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/A-cabin-pinouts.xlsx
+++ b/docs/harness/wirelist/A-cabin-pinouts.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ECU-A (ecu_a)'!$A$2:$D$36</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'ECU-A (ecu_a)'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BULKHEAD (bh_a_fw)'!$A$2:$D$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BULKHEAD (bh_a_fw)'!$A$2:$D$71</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'BULKHEAD (bh_a_fw)'!$1:$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'FRONT WS INLINE (ix_ws_front_p)'!$A$2:$D$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'FRONT WS INLINE (ix_ws_front_p)'!$1:$2</definedName>
@@ -582,7 +582,7 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 34</t>
+          <t>BULKHEAD pin 24</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 33</t>
+          <t>BULKHEAD pin 23</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 32</t>
+          <t>BULKHEAD pin 22</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 31</t>
+          <t>BULKHEAD pin 21</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 9</t>
+          <t>BULKHEAD pin 74</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 38</t>
+          <t>BULKHEAD pin 12</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 37</t>
+          <t>BULKHEAD pin 11</t>
         </is>
       </c>
     </row>
@@ -824,7 +824,7 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 36</t>
+          <t>BULKHEAD pin 10</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 35</t>
+          <t>BULKHEAD pin 9</t>
         </is>
       </c>
     </row>
@@ -890,7 +890,7 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 40</t>
+          <t>BULKHEAD pin 70</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 41</t>
+          <t>BULKHEAD pin 33</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 30</t>
+          <t>BULKHEAD pin 17</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 39</t>
+          <t>BULKHEAD pin 58</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 24</t>
+          <t>BULKHEAD pin 42</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 44</t>
+          <t>BULKHEAD pin 84</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 17</t>
+          <t>BULKHEAD pin 53</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 21</t>
+          <t>BULKHEAD pin 31</t>
         </is>
       </c>
     </row>
@@ -1286,7 +1286,7 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 25</t>
+          <t>BULKHEAD pin 44</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1369,17 +1369,17 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>w_inj_pwr_ac</t>
+          <t>w_cop_pwr_ac</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Injector +12 V feed</t>
+          <t>Coil +12 V feed</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>FB-LOGIC pin BUS2-4</t>
+          <t>FB-LOGIC pin BUS2-3</t>
         </is>
       </c>
     </row>
@@ -1389,723 +1389,611 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>w_cop_pwr_ac</t>
+          <t>w_inj_pwr_ac</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Coil +12 V feed</t>
+          <t>Injector +12 V feed</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>FB-LOGIC pin BUS2-3</t>
+          <t>FB-LOGIC pin BUS2-4</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>w200_c</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr"/>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Crank sensor signal</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>ECU-A pin A8</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>w_gnd_a_c41</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr"/>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Gnd crank sensor</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>SENSOR GND BUS pin 3</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>w_shc_crank</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr"/>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Crank sensor shield</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>w_rail_sp_8v_c</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr"/>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>+8 V to cam sensor</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>splice sp_8v (SP-8V: +8 V cam sensor supply)</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>w_cam_sig_c</t>
-        </is>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr"/>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Cam sensor signal</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>splice sp_trig2 (SP-CAM: cam signal + 1.8k pull-up to +8V)</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
-        <v>14</v>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>w_gnd_a_c42</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr"/>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Gnd cam sensor</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>SENSOR GND BUS pin 4</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>w_shc_cam</t>
+          <t>w120_c</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Cam sensor shield</t>
+          <t>Coil 1 trigger (IGT)</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>ECU-A pin A13</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>w_5v_a_c40</t>
+          <t>w121_c</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>+5 V turbo speed</t>
+          <t>Coil 2 trigger (IGT)</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>+5V BUS pin 4</t>
+          <t>ECU-A pin A12</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>w16_c</t>
+          <t>w122_c</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Turbo speed signal</t>
+          <t>Coil 3 trigger (IGT)</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>ECU-A pin A30</t>
+          <t>ECU-A pin A11</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>w_gnd_a_c43</t>
+          <t>w123_c</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Gnd turbo speed</t>
+          <t>Coil 4 trigger (IGT)</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>SENSOR GND BUS pin 5</t>
+          <t>ECU-A pin A10</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>w_shc_turbo</t>
+          <t>w_5v_brail_c46</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Turbo speed shield</t>
+          <t>+5 V fuel pressure</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>+5V BUS pin 6</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>w_rail_sp_sw12_c</t>
+          <t>w_5v_a_c39</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>+12 V boost + flex</t>
+          <t>+5 V MAP sensor</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>splice sp_sw12 (SP-SW12: switched +12 V)</t>
+          <t>+5V BUS pin 3</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>w48_c</t>
+          <t>w26_c</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Flex fuel signal</t>
+          <t>MAP sensor signal</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>ECU-A pin A31</t>
+          <t>ECU-A pin A17</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>w_shc_flex</t>
+          <t>w_gnd_a_c44</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Flex fuel shield</t>
+          <t>Gnd flex + MAP</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>SENSOR GND BUS pin 6</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>23</v>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>w_rail_sp_5v_c</t>
-        </is>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr"/>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>+5 V throttle sensor</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>+5V BUS pin 2</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n">
-        <v>24</v>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>w128_c</t>
-        </is>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="B20" s="8" t="inlineStr"/>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Throttle pos 1 main</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>ECU-A pin A22</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>w129_c</t>
+          <t>w108_c</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Throttle pos 2 sub</t>
+          <t>Injector 1 drive (-)</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>ECU-A pin A33</t>
+          <t>ECU-A pin A4</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>w_rail_sp_gndout_c</t>
+          <t>w109_c</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Gnd IAT/TPS/coolant</t>
+          <t>Injector 2 drive (-)</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>SENSOR GND BUS pin 2</t>
+          <t>ECU-A pin A3</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>w_shc_etbs</t>
+          <t>w110_c</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Throttle shield</t>
+          <t>Injector 3 drive (-)</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+          <t>ECU-A pin A2</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>w_5v_a_c39</t>
+          <t>w111_c</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>+5 V MAP sensor</t>
+          <t>Injector 4 drive (-)</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>+5V BUS pin 3</t>
+          <t>ECU-A pin A1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>w_gnd_a_c44</t>
+          <t>w_5v_brail_c47</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Gnd flex + MAP</t>
+          <t>+5 V coolant press</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>SENSOR GND BUS pin 6</t>
+          <t>+5V BUS pin 7</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>w26_c</t>
+          <t>w_5v_brail_c45</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>MAP sensor signal</t>
+          <t>+5 V oil pressure</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>ECU-A pin A17</t>
+          <t>+5V BUS pin 5</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>w108_c</t>
+          <t>w_rail_sp_sw12_c</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Injector 1 drive (-)</t>
+          <t>+12 V boost + flex</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>ECU-A pin A4</t>
+          <t>splice sp_sw12 (SP-SW12: switched +12 V)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>w109_c</t>
+          <t>w48_c</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Injector 2 drive (-)</t>
+          <t>Flex fuel signal</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>ECU-A pin A3</t>
+          <t>ECU-A pin A31</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>w110_c</t>
+          <t>w_shc_flex</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Injector 3 drive (-)</t>
+          <t>Flex fuel shield</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>ECU-A pin A2</t>
+          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>w111_c</t>
+          <t>w202_c</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>Injector 4 drive (-)</t>
+          <t>Intake temp signal</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>ECU-A pin A1</t>
+          <t>ECU-A pin A16</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>w120_c</t>
+          <t>w_rail_sp_gndout_c</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Coil 1 trigger (IGT)</t>
+          <t>Gnd IAT/TPS/coolant</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>ECU-A pin A13</t>
+          <t>SENSOR GND BUS pin 2</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="n">
-        <v>36</v>
-      </c>
-      <c r="B32" s="8" t="inlineStr">
-        <is>
-          <t>w121_c</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="B32" s="8" t="inlineStr"/>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Coil 2 trigger (IGT)</t>
-        </is>
-      </c>
-      <c r="D32" s="10" t="inlineStr">
-        <is>
-          <t>ECU-A pin A12</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n">
-        <v>37</v>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>w122_c</t>
-        </is>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="B33" s="5" t="inlineStr"/>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Coil 3 trigger (IGT)</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>ECU-A pin A11</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="n">
-        <v>38</v>
-      </c>
-      <c r="B34" s="8" t="inlineStr">
-        <is>
-          <t>w123_c</t>
-        </is>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="B34" s="8" t="inlineStr"/>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>Coil 4 trigger (IGT)</t>
-        </is>
-      </c>
-      <c r="D34" s="10" t="inlineStr">
-        <is>
-          <t>ECU-A pin A10</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
-        <v>39</v>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>w103_c</t>
-        </is>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="B35" s="5" t="inlineStr"/>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Boost solenoid (-)</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>ECU-A pin A21</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>w201_c</t>
-        </is>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="B36" s="8" t="inlineStr"/>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>Coolant temp signal</t>
-        </is>
-      </c>
-      <c r="D36" s="10" t="inlineStr">
-        <is>
-          <t>ECU-A pin A15</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n">
-        <v>41</v>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>w202_c</t>
-        </is>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="B37" s="5" t="inlineStr"/>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Intake temp signal</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>ECU-A pin A16</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>w_fb_mrs_en</t>
+          <t>w_rail_sp_5v_c</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>EHPS enable +12 V</t>
+          <t>+5 V throttle sensor</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>FB-LOGIC pin BUS2-12</t>
+          <t>+5V BUS pin 2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>w_mrs_c</t>
+          <t>w128_c</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>EHPS pump speed</t>
+          <t>Throttle pos 1 main</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>ECU-A pin A27</t>
+          <t>ECU-A pin A22</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B40" s="8" t="inlineStr"/>
       <c r="C40" s="9" t="inlineStr">
@@ -2117,15 +2005,23 @@
     </row>
     <row r="41">
       <c r="A41" s="5" t="n">
-        <v>46</v>
-      </c>
-      <c r="B41" s="5" t="inlineStr"/>
+        <v>44</v>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>w129_c</t>
+        </is>
+      </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>spare, sealing plug</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr"/>
+          <t>Throttle pos 2 sub</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>ECU-A pin A33</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="n">
@@ -2133,107 +2029,99 @@
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>w_5v_brail_c45</t>
+          <t>w_shc_etbs</t>
         </is>
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>+5 V oil pressure</t>
+          <t>Throttle shield</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>+5V BUS pin 5</t>
+          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n">
-        <v>50</v>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>w_5v_brail_c46</t>
-        </is>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr"/>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>+5 V fuel pressure</t>
-        </is>
-      </c>
-      <c r="D43" s="7" t="inlineStr">
-        <is>
-          <t>+5V BUS pin 6</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="8" t="n">
-        <v>51</v>
-      </c>
-      <c r="B44" s="8" t="inlineStr">
-        <is>
-          <t>w_5v_brail_c47</t>
-        </is>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="B44" s="8" t="inlineStr"/>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>+5 V coolant press</t>
-        </is>
-      </c>
-      <c r="D44" s="10" t="inlineStr">
-        <is>
-          <t>+5V BUS pin 7</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n">
         <v>52</v>
       </c>
-      <c r="B45" s="5" t="inlineStr"/>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>w_5v_a_c40</t>
+        </is>
+      </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>spare, sealing plug</t>
-        </is>
-      </c>
-      <c r="D45" s="7" t="inlineStr"/>
+          <t>+5 V turbo speed</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>+5V BUS pin 4</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="n">
         <v>53</v>
       </c>
-      <c r="B46" s="8" t="inlineStr"/>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>w16_c</t>
+        </is>
+      </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>spare, sealing plug</t>
-        </is>
-      </c>
-      <c r="D46" s="10" t="inlineStr"/>
+          <t>Turbo speed signal</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>ECU-A pin A30</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n">
-        <v>56</v>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>w_eps_rly</t>
-        </is>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr"/>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>EHPS relay coil (-)</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>EHPS RELAY pin 85</t>
-        </is>
-      </c>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B48" s="8" t="inlineStr"/>
       <c r="C48" s="9" t="inlineStr">
@@ -2245,42 +2133,394 @@
     </row>
     <row r="49">
       <c r="A49" s="5" t="n">
-        <v>58</v>
-      </c>
-      <c r="B49" s="5" t="inlineStr"/>
+        <v>56</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>w_gnd_a_c43</t>
+        </is>
+      </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>spare, sealing plug</t>
-        </is>
-      </c>
-      <c r="D49" s="7" t="inlineStr"/>
+          <t>Gnd turbo speed</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>SENSOR GND BUS pin 5</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="n">
-        <v>59</v>
-      </c>
-      <c r="B50" s="8" t="inlineStr"/>
+        <v>57</v>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>w_shc_turbo</t>
+        </is>
+      </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>spare, sealing plug</t>
-        </is>
-      </c>
-      <c r="D50" s="10" t="inlineStr"/>
+          <t>Turbo speed shield</t>
+        </is>
+      </c>
+      <c r="D50" s="10" t="inlineStr">
+        <is>
+          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n">
-        <v>61</v>
-      </c>
-      <c r="B51" s="5" t="inlineStr"/>
+        <v>58</v>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>w103_c</t>
+        </is>
+      </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
+          <t>Boost solenoid (-)</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>ECU-A pin A21</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="n">
+        <v>63</v>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>w_rail_sp_8v_c</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>+8 V to cam sensor</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>splice sp_8v (SP-8V: +8 V cam sensor supply)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>w_cam_sig_c</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Cam sensor signal</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>splice sp_trig2 (SP-CAM: cam signal + 1.8k pull-up to +8V)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>w_gnd_a_c42</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>Gnd cam sensor</t>
+        </is>
+      </c>
+      <c r="D54" s="10" t="inlineStr">
+        <is>
+          <t>SENSOR GND BUS pin 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>w_shc_cam</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Cam sensor shield</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>w201_c</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>Coolant temp signal</t>
+        </is>
+      </c>
+      <c r="D56" s="10" t="inlineStr">
+        <is>
+          <t>ECU-A pin A15</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>w200_c</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Crank sensor signal</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>ECU-A pin A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="n">
+        <v>75</v>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>w_gnd_a_c41</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
+        <is>
+          <t>Gnd crank sensor</t>
+        </is>
+      </c>
+      <c r="D58" s="10" t="inlineStr">
+        <is>
+          <t>SENSOR GND BUS pin 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>w_shc_crank</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>Crank sensor shield</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>splice sp_shield_a (SP-SHIELD-A: shield drains)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>w_fb_mrs_en</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>EHPS enable +12 V</t>
+        </is>
+      </c>
+      <c r="D60" s="10" t="inlineStr">
+        <is>
+          <t>FB-LOGIC pin BUS2-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="n">
+        <v>84</v>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>w_mrs_c</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>EHPS pump speed</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>ECU-A pin A27</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>w_eps_rly</t>
+        </is>
+      </c>
+      <c r="C62" s="9" t="inlineStr">
+        <is>
+          <t>EHPS relay coil (-)</t>
+        </is>
+      </c>
+      <c r="D62" s="10" t="inlineStr">
+        <is>
+          <t>EHPS RELAY pin 85</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="n">
+        <v>86</v>
+      </c>
+      <c r="B63" s="5" t="inlineStr"/>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
           <t>spare, sealing plug</t>
         </is>
       </c>
-      <c r="D51" s="7" t="inlineStr"/>
+      <c r="D63" s="7" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="B64" s="8" t="inlineStr"/>
+      <c r="C64" s="9" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D64" s="10" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="n">
+        <v>88</v>
+      </c>
+      <c r="B65" s="5" t="inlineStr"/>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="B66" s="8" t="inlineStr"/>
+      <c r="C66" s="9" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D66" s="10" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="B67" s="5" t="inlineStr"/>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="B68" s="8" t="inlineStr"/>
+      <c r="C68" s="9" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D68" s="10" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="n">
+        <v>92</v>
+      </c>
+      <c r="B69" s="5" t="inlineStr"/>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="B70" s="8" t="inlineStr"/>
+      <c r="C70" s="9" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D70" s="10" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="n">
+        <v>94</v>
+      </c>
+      <c r="B71" s="5" t="inlineStr"/>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>spare, sealing plug</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:D51"/>
+  <autoFilter ref="A2:D71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -2700,7 +2940,7 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 23</t>
+          <t>BULKHEAD pin 41</t>
         </is>
       </c>
     </row>
@@ -2720,7 +2960,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 28</t>
+          <t>BULKHEAD pin 16</t>
         </is>
       </c>
     </row>
@@ -2740,7 +2980,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 16</t>
+          <t>BULKHEAD pin 52</t>
         </is>
       </c>
     </row>
@@ -2760,7 +3000,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 47</t>
+          <t>BULKHEAD pin 27</t>
         </is>
       </c>
     </row>
@@ -2780,7 +3020,7 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 50</t>
+          <t>BULKHEAD pin 13</t>
         </is>
       </c>
     </row>
@@ -2800,7 +3040,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 51</t>
+          <t>BULKHEAD pin 25</t>
         </is>
       </c>
     </row>
@@ -2903,7 +3143,7 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 26</t>
+          <t>BULKHEAD pin 34</t>
         </is>
       </c>
     </row>
@@ -2923,7 +3163,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 10</t>
+          <t>BULKHEAD pin 75</t>
         </is>
       </c>
     </row>
@@ -2943,7 +3183,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 14</t>
+          <t>BULKHEAD pin 65</t>
         </is>
       </c>
     </row>
@@ -2963,7 +3203,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 18</t>
+          <t>BULKHEAD pin 56</t>
         </is>
       </c>
     </row>
@@ -2983,7 +3223,7 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>BULKHEAD pin 29</t>
+          <t>BULKHEAD pin 18</t>
         </is>
       </c>
     </row>

</xml_diff>